<commit_message>
Verify PL and EFL points deductions against dragonfootball.co.uk
Adds four missing deductions, corrects Reading 2023/24 to -6, and marks every
PL/EFL deduction as verified. National League ones stay marked check.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S5Qc48tZkYoqs3XftGiQZ8
</commit_message>
<xml_diff>
--- a/data/processed/real_tables.xlsx
+++ b/data/processed/real_tables.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4939" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4955" uniqueCount="272">
   <si>
     <t>season</t>
   </si>
@@ -627,28 +627,19 @@
     <t>confidence</t>
   </si>
   <si>
-    <t>chester_city</t>
+    <t>stockport_county</t>
   </si>
   <si>
-    <t>bury</t>
+    <t>bournemouth</t>
   </si>
   <si>
-    <t>dover_athletic</t>
-  </si>
-  <si>
-    <t>stockport_county</t>
+    <t>darlington</t>
   </si>
   <si>
     <t>luton_town</t>
   </si>
   <si>
-    <t>bournemouth</t>
-  </si>
-  <si>
     <t>rotherham_united</t>
-  </si>
-  <si>
-    <t>darlington</t>
   </si>
   <si>
     <t>portsmouth</t>
@@ -657,13 +648,16 @@
     <t>crystal_palace</t>
   </si>
   <si>
+    <t>hartlepool_united</t>
+  </si>
+  <si>
     <t>southampton</t>
   </si>
   <si>
-    <t>hartlepool_united</t>
+    <t>salisbury_city</t>
   </si>
   <si>
-    <t>salisbury_city</t>
+    <t>chester_city</t>
   </si>
   <si>
     <t>plymouth_argyle</t>
@@ -675,10 +669,16 @@
     <t>torquay_united</t>
   </si>
   <si>
+    <t>kidderminster_harriers</t>
+  </si>
+  <si>
     <t>port_vale</t>
   </si>
   <si>
     <t>coventry_city</t>
+  </si>
+  <si>
+    <t>aldershot_town</t>
   </si>
   <si>
     <t>afc_wimbledon</t>
@@ -693,7 +693,16 @@
     <t>bolton_wanderers</t>
   </si>
   <si>
+    <t>bury</t>
+  </si>
+  <si>
+    <t>macclesfield_town</t>
+  </si>
+  <si>
     <t>sheffield_wednesday</t>
+  </si>
+  <si>
+    <t>dover_athletic</t>
   </si>
   <si>
     <t>derby_county</t>
@@ -708,58 +717,73 @@
     <t>nottingham_forest</t>
   </si>
   <si>
-    <t>kidderminster_harriers</t>
-  </si>
-  <si>
-    <t>aldershot_town</t>
-  </si>
-  <si>
-    <t>macclesfield_town</t>
+    <t>morecambe</t>
   </si>
   <si>
     <t>southend_united</t>
   </si>
   <si>
+    <t>sheffield_united</t>
+  </si>
+  <si>
     <t>leicester_city</t>
+  </si>
+  <si>
+    <t>west_bromwich_albion</t>
   </si>
   <si>
     <t>expunged</t>
   </si>
   <si>
+    <t>Administration</t>
+  </si>
+  <si>
+    <t>Exit from administration without a CVA</t>
+  </si>
+  <si>
+    <t>10 administration + 20 Football League/FA irregularities</t>
+  </si>
+  <si>
+    <t>Fielded an ineligible player</t>
+  </si>
+  <si>
+    <t>Administration (parent company)</t>
+  </si>
+  <si>
+    <t>Administration (also demoted two divisions at season end)</t>
+  </si>
+  <si>
     <t>Expelled by the Conference in Feb 2010; record expunged</t>
+  </si>
+  <si>
+    <t>Financial irregularities (from memory; not yet verified)</t>
+  </si>
+  <si>
+    <t>Administration (also demoted four divisions at season end)</t>
+  </si>
+  <si>
+    <t>Administration (applied to 2012/13 by the EFL; already bottom)</t>
+  </si>
+  <si>
+    <t>Insolvency event (CVA not agreed)</t>
+  </si>
+  <si>
+    <t>Administration (entered May 2013; applied to 2013/14)</t>
+  </si>
+  <si>
+    <t>Breach of EFL profitability and sustainability rules</t>
   </si>
   <si>
     <t>Expelled from the EFL in Aug 2019 before playing; League One ran with 23 clubs</t>
   </si>
   <si>
-    <t>Refused to play after Jan 2021; record expunged (12-point deduction carried into 2021/22)</t>
-  </si>
-  <si>
-    <t>Administration</t>
-  </si>
-  <si>
-    <t>10 administration + 20 Football League/FA irregularities</t>
-  </si>
-  <si>
-    <t>Exit from administration without a CVA</t>
-  </si>
-  <si>
-    <t>Administration (parent company)</t>
-  </si>
-  <si>
-    <t>Fielded an ineligible player</t>
-  </si>
-  <si>
-    <t>Administration (also demoted two divisions at season end)</t>
-  </si>
-  <si>
-    <t>Insolvency event (CVA not agreed)</t>
-  </si>
-  <si>
-    <t>Breach of EFL profitability and sustainability rules</t>
+    <t>Unpaid wages and fixture failures (total after the July 2020 appeal ruling)</t>
   </si>
   <si>
     <t>Breach of profitability and sustainability rules (12 reduced to 6 on appeal)</t>
+  </si>
+  <si>
+    <t>Refused to play after Jan 2021; record expunged (12-point deduction carried into 2021/22)</t>
   </si>
   <si>
     <t>12 administration + 9 profitability and sustainability</t>
@@ -774,34 +798,28 @@
     <t>Breach of business plan agreed with the EFL</t>
   </si>
   <si>
+    <t>Failure to pay players on time</t>
+  </si>
+  <si>
     <t>Breaches of PL profitability and sustainability rules (10 cut to 6 on appeal; then 2 more)</t>
   </si>
   <si>
     <t>Breach of PL profitability and sustainability rules</t>
   </si>
   <si>
-    <t>Financial irregularities (from memory; not yet verified)</t>
-  </si>
-  <si>
-    <t>Administration (also demoted four divisions at season end)</t>
-  </si>
-  <si>
-    <t>Administration (entered May 2013; applied to 2013/14)</t>
-  </si>
-  <si>
-    <t>Unpaid wages and fixture failures (total after the July 2020 appeal ruling)</t>
-  </si>
-  <si>
-    <t>Failure to pay players on time</t>
+    <t>Late wages and late tax payments</t>
   </si>
   <si>
     <t>Failure to pay players on time (applied at the start of 2023/24)</t>
   </si>
   <si>
-    <t>Failures to pay players and HMRC on time</t>
+    <t>Late payment of player wages (suspended deduction activated)</t>
   </si>
   <si>
     <t>Failure to pay HMRC and players (from memory; not yet verified)</t>
+  </si>
+  <si>
+    <t>Late transfer payments to other clubs</t>
   </si>
   <si>
     <t>Breach of profitability and sustainability rules (2023/24 accounts)</t>
@@ -810,10 +828,13 @@
     <t>12 administration + 6 payment failures (from memory; not yet verified)</t>
   </si>
   <si>
-    <t>high</t>
+    <t>verified</t>
   </si>
   <si>
     <t>check</t>
+  </si>
+  <si>
+    <t>high</t>
   </si>
 </sst>
 </file>
@@ -34621,13 +34642,13 @@
         <v>92</v>
       </c>
       <c r="L388">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M388">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="N388">
-        <v>2</v>
+        <v>1.956522</v>
       </c>
     </row>
     <row r="389" spans="1:15">
@@ -36375,7 +36396,7 @@
         <v>19</v>
       </c>
       <c r="C428" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="D428">
         <v>46</v>
@@ -36390,13 +36411,13 @@
         <v>19</v>
       </c>
       <c r="H428">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="I428">
         <v>58</v>
       </c>
       <c r="J428">
-        <v>-10</v>
+        <v>-14</v>
       </c>
       <c r="K428">
         <v>53</v>
@@ -36419,7 +36440,7 @@
         <v>20</v>
       </c>
       <c r="C429" t="s">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="D429">
         <v>46</v>
@@ -36428,31 +36449,31 @@
         <v>13</v>
       </c>
       <c r="F429">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G429">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H429">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I429">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="J429">
         <v>-14</v>
       </c>
       <c r="K429">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L429">
         <v>0</v>
       </c>
       <c r="M429">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N429">
-        <v>1.152174</v>
+        <v>1.130435</v>
       </c>
     </row>
     <row r="430" spans="1:15">
@@ -36463,7 +36484,7 @@
         <v>21</v>
       </c>
       <c r="C430" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D430">
         <v>46</v>
@@ -36472,31 +36493,31 @@
         <v>13</v>
       </c>
       <c r="F430">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G430">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H430">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="I430">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J430">
-        <v>-14</v>
+        <v>-10</v>
       </c>
       <c r="K430">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L430">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M430">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="N430">
-        <v>1.130435</v>
+        <v>1.108696</v>
       </c>
     </row>
     <row r="431" spans="1:15">
@@ -53482,40 +53503,40 @@
         <v>16</v>
       </c>
       <c r="C376" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="D376">
         <v>46</v>
       </c>
       <c r="E376">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F376">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="G376">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H376">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I376">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J376">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="K376">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="L376">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M376">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="N376">
-        <v>1.195652</v>
+        <v>1.152174</v>
       </c>
     </row>
     <row r="377" spans="1:15">
@@ -53526,34 +53547,34 @@
         <v>17</v>
       </c>
       <c r="C377" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="D377">
         <v>46</v>
       </c>
       <c r="E377">
+        <v>16</v>
+      </c>
+      <c r="F377">
         <v>11</v>
       </c>
-      <c r="F377">
-        <v>20</v>
-      </c>
       <c r="G377">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="H377">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I377">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J377">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="K377">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="L377">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M377">
         <v>53</v>
@@ -61451,13 +61472,13 @@
         <v>48</v>
       </c>
       <c r="L121">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M121">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="N121">
-        <v>1.043478</v>
+        <v>0.826087</v>
       </c>
       <c r="O121" t="s">
         <v>76</v>
@@ -72866,13 +72887,13 @@
         <v>61</v>
       </c>
       <c r="L376">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M376">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="N376">
-        <v>1.326087</v>
+        <v>1.26087</v>
       </c>
     </row>
     <row r="377" spans="1:15">
@@ -94639,7 +94660,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -94667,62 +94688,71 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
         <v>202</v>
       </c>
       <c r="D2" t="s">
-        <v>234</v>
+        <v>11</v>
+      </c>
+      <c r="E2">
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="G2" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3">
-        <v>2019</v>
+        <v>2008</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
         <v>203</v>
       </c>
       <c r="D3" t="s">
-        <v>147</v>
+        <v>11</v>
+      </c>
+      <c r="E3">
+        <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G3" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4">
-        <v>2020</v>
+        <v>2008</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
         <v>204</v>
       </c>
       <c r="D4" t="s">
-        <v>234</v>
+        <v>11</v>
+      </c>
+      <c r="E4">
+        <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G4" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -94730,7 +94760,7 @@
         <v>2008</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
         <v>205</v>
@@ -94739,13 +94769,13 @@
         <v>11</v>
       </c>
       <c r="E5">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G5" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -94762,21 +94792,21 @@
         <v>11</v>
       </c>
       <c r="E6">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
         <v>239</v>
       </c>
       <c r="G6" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C7" t="s">
         <v>207</v>
@@ -94785,21 +94815,21 @@
         <v>11</v>
       </c>
       <c r="E7">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="G7" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="B8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C8" t="s">
         <v>208</v>
@@ -94808,21 +94838,21 @@
         <v>11</v>
       </c>
       <c r="E8">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="G8" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="B9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" t="s">
         <v>209</v>
@@ -94831,13 +94861,13 @@
         <v>11</v>
       </c>
       <c r="E9">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G9" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -94845,7 +94875,7 @@
         <v>2009</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" t="s">
         <v>210</v>
@@ -94854,13 +94884,13 @@
         <v>11</v>
       </c>
       <c r="E10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F10" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="G10" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -94868,7 +94898,7 @@
         <v>2009</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C11" t="s">
         <v>211</v>
@@ -94880,10 +94910,10 @@
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="G11" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -94891,27 +94921,24 @@
         <v>2009</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C12" t="s">
         <v>212</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12">
-        <v>10</v>
+        <v>237</v>
       </c>
       <c r="F12" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="G12" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="B13">
         <v>3</v>
@@ -94923,21 +94950,21 @@
         <v>11</v>
       </c>
       <c r="E13">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F13" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="G13" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="B14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C14" t="s">
         <v>214</v>
@@ -94946,13 +94973,13 @@
         <v>11</v>
       </c>
       <c r="E14">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="G14" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -94960,7 +94987,7 @@
         <v>2010</v>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" t="s">
         <v>215</v>
@@ -94969,13 +94996,13 @@
         <v>11</v>
       </c>
       <c r="E15">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G15" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -94983,7 +95010,7 @@
         <v>2010</v>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16" t="s">
         <v>216</v>
@@ -94992,36 +95019,36 @@
         <v>11</v>
       </c>
       <c r="E16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F16" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="G16" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F17" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="G17" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -95029,10 +95056,10 @@
         <v>2011</v>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -95044,7 +95071,7 @@
         <v>238</v>
       </c>
       <c r="G18" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -95052,10 +95079,10 @@
         <v>2011</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -95064,10 +95091,10 @@
         <v>10</v>
       </c>
       <c r="F19" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="G19" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -95078,7 +95105,7 @@
         <v>3</v>
       </c>
       <c r="C20" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
@@ -95090,7 +95117,7 @@
         <v>238</v>
       </c>
       <c r="G20" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -95101,7 +95128,7 @@
         <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
@@ -95113,15 +95140,15 @@
         <v>238</v>
       </c>
       <c r="G21" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" t="s">
         <v>219</v>
@@ -95133,10 +95160,10 @@
         <v>10</v>
       </c>
       <c r="F22" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="G22" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -95144,33 +95171,33 @@
         <v>2013</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="G23" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
@@ -95179,176 +95206,173 @@
         <v>3</v>
       </c>
       <c r="F24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G24" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25">
-        <v>2018</v>
+        <v>2013</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D25" t="s">
         <v>11</v>
       </c>
       <c r="E25">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="G25" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="B26">
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F26" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G26" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="B27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F27" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="G27" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F28" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="G28" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F29" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="G29" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="B30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C30" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D30" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30">
-        <v>6</v>
+        <v>147</v>
       </c>
       <c r="F30" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G30" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="B31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C31" t="s">
-        <v>204</v>
+        <v>225</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F31" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G31" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="B32">
         <v>2</v>
@@ -95363,41 +95387,38 @@
         <v>6</v>
       </c>
       <c r="F32" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="G32" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="B33">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C33" t="s">
         <v>227</v>
       </c>
       <c r="D33" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33">
-        <v>8</v>
+        <v>237</v>
       </c>
       <c r="F33" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G33" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="B34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="s">
         <v>228</v>
@@ -95406,21 +95427,21 @@
         <v>11</v>
       </c>
       <c r="E34">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="F34" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G34" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35">
-        <v>2010</v>
+        <v>2021</v>
       </c>
       <c r="B35">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C35" t="s">
         <v>229</v>
@@ -95429,105 +95450,105 @@
         <v>11</v>
       </c>
       <c r="E35">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F35" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="G35" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36">
-        <v>2011</v>
+        <v>2021</v>
       </c>
       <c r="B36">
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>209</v>
+        <v>227</v>
       </c>
       <c r="D36" t="s">
         <v>11</v>
       </c>
       <c r="E36">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F36" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="G36" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37">
-        <v>2013</v>
+        <v>2022</v>
       </c>
       <c r="B37">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C37" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F37" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G37" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="38" spans="1:7">
       <c r="A38">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="B38">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="F38" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="G38" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F39" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="G39" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -95535,22 +95556,22 @@
         <v>2023</v>
       </c>
       <c r="B40">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F40" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="G40" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -95561,19 +95582,19 @@
         <v>3</v>
       </c>
       <c r="C41" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="E41">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F41" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G41" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -95581,68 +95602,160 @@
         <v>2023</v>
       </c>
       <c r="B42">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C42" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F42" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G42" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="43" spans="1:7">
       <c r="A43">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C43" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
       </c>
       <c r="E43">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F43" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G43" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B44">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C44" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
       </c>
       <c r="E44">
+        <v>10</v>
+      </c>
+      <c r="F44" t="s">
+        <v>265</v>
+      </c>
+      <c r="G44" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45">
+        <v>2024</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+      <c r="C45" t="s">
+        <v>234</v>
+      </c>
+      <c r="D45" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45" t="s">
+        <v>266</v>
+      </c>
+      <c r="G45" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46">
+        <v>2025</v>
+      </c>
+      <c r="B46">
+        <v>2</v>
+      </c>
+      <c r="C46" t="s">
+        <v>235</v>
+      </c>
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46">
+        <v>6</v>
+      </c>
+      <c r="F46" t="s">
+        <v>267</v>
+      </c>
+      <c r="G46" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47">
+        <v>2025</v>
+      </c>
+      <c r="B47">
+        <v>2</v>
+      </c>
+      <c r="C47" t="s">
+        <v>226</v>
+      </c>
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47">
         <v>18</v>
       </c>
-      <c r="F44" t="s">
-        <v>262</v>
-      </c>
-      <c r="G44" t="s">
-        <v>264</v>
+      <c r="F47" t="s">
+        <v>268</v>
+      </c>
+      <c r="G47" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48">
+        <v>2025</v>
+      </c>
+      <c r="B48">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>236</v>
+      </c>
+      <c r="D48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48">
+        <v>2</v>
+      </c>
+      <c r="F48" t="s">
+        <v>256</v>
+      </c>
+      <c r="G48" t="s">
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Source every deduction and check all tables against Wikipedia
National League deductions now come from the Wikipedia final tables instead
of memory. Adds Crystal Palace 2008/09 and Bury 2015/16 deductions, removes
Aldershot 2012/13, records a source per adjustment, and adds a test that every
position and points total matches the published tables.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S5Qc48tZkYoqs3XftGiQZ8
</commit_message>
<xml_diff>
--- a/data/processed/real_tables.xlsx
+++ b/data/processed/real_tables.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4955" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5023" uniqueCount="291">
   <si>
     <t>season</t>
   </si>
@@ -624,7 +624,10 @@
     <t>reason</t>
   </si>
   <si>
-    <t>confidence</t>
+    <t>source</t>
+  </si>
+  <si>
+    <t>crystal_palace</t>
   </si>
   <si>
     <t>stockport_county</t>
@@ -642,16 +645,28 @@
     <t>rotherham_united</t>
   </si>
   <si>
-    <t>portsmouth</t>
+    <t>crawley_town</t>
   </si>
   <si>
-    <t>crystal_palace</t>
+    <t>mansfield_town</t>
+  </si>
+  <si>
+    <t>oxford_united</t>
+  </si>
+  <si>
+    <t>portsmouth</t>
   </si>
   <si>
     <t>hartlepool_united</t>
   </si>
   <si>
     <t>southampton</t>
+  </si>
+  <si>
+    <t>gateshead</t>
+  </si>
+  <si>
+    <t>grays_athletic</t>
   </si>
   <si>
     <t>salisbury_city</t>
@@ -669,7 +684,16 @@
     <t>torquay_united</t>
   </si>
   <si>
+    <t>histon</t>
+  </si>
+  <si>
+    <t>kettering_town</t>
+  </si>
+  <si>
     <t>kidderminster_harriers</t>
+  </si>
+  <si>
+    <t>rushden_and_diamonds</t>
   </si>
   <si>
     <t>port_vale</t>
@@ -678,22 +702,37 @@
     <t>coventry_city</t>
   </si>
   <si>
+    <t>afc_wimbledon</t>
+  </si>
+  <si>
     <t>aldershot_town</t>
   </si>
   <si>
-    <t>afc_wimbledon</t>
+    <t>alfreton_town</t>
+  </si>
+  <si>
+    <t>afc_telford_united</t>
+  </si>
+  <si>
+    <t>forest_green_rovers</t>
+  </si>
+  <si>
+    <t>nuneaton_borough</t>
+  </si>
+  <si>
+    <t>bury</t>
   </si>
   <si>
     <t>birmingham_city</t>
+  </si>
+  <si>
+    <t>braintree_town</t>
   </si>
   <si>
     <t>wigan_athletic</t>
   </si>
   <si>
     <t>bolton_wanderers</t>
-  </si>
-  <si>
-    <t>bury</t>
   </si>
   <si>
     <t>macclesfield_town</t>
@@ -735,6 +774,9 @@
     <t>expunged</t>
   </si>
   <si>
+    <t>Fielded an ineligible player</t>
+  </si>
+  <si>
     <t>Administration</t>
   </si>
   <si>
@@ -744,34 +786,49 @@
     <t>10 administration + 20 Football League/FA irregularities</t>
   </si>
   <si>
-    <t>Fielded an ineligible player</t>
+    <t>Points deducted, cut on appeal (only BBC reference titles on the page give the cause)</t>
+  </si>
+  <si>
+    <t>Points deduction (only BBC reference titles on the page give the cause)</t>
+  </si>
+  <si>
+    <t>Fielded an ineligible player (BBC: "Five-point deduction for Oxford")</t>
   </si>
   <si>
     <t>Administration (parent company)</t>
   </si>
   <si>
-    <t>Administration (also demoted two divisions at season end)</t>
+    <t>Failed to fulfil a fixture</t>
+  </si>
+  <si>
+    <t>Fielded ineligible players</t>
+  </si>
+  <si>
+    <t>Administration (also demoted at season end)</t>
   </si>
   <si>
     <t>Expelled by the Conference in Feb 2010; record expunged</t>
   </si>
   <si>
-    <t>Financial irregularities (from memory; not yet verified)</t>
+    <t>Submitted misleading financial information</t>
   </si>
   <si>
-    <t>Administration (also demoted four divisions at season end)</t>
+    <t>Submitted misleading financial information (expelled after the season)</t>
   </si>
   <si>
-    <t>Administration (applied to 2012/13 by the EFL; already bottom)</t>
+    <t>Failed to pay football creditors</t>
   </si>
   <si>
     <t>Insolvency event (CVA not agreed)</t>
   </si>
   <si>
-    <t>Administration (entered May 2013; applied to 2013/14)</t>
+    <t>Fielded an unregistered player</t>
   </si>
   <si>
     <t>Breach of EFL profitability and sustainability rules</t>
+  </si>
+  <si>
+    <t>Breach of financial regulations (also demoted at season end)</t>
   </si>
   <si>
     <t>Expelled from the EFL in Aug 2019 before playing; League One ran with 23 clubs</t>
@@ -792,13 +849,16 @@
     <t>Breach of profitability and sustainability rules</t>
   </si>
   <si>
-    <t>Carried over from 2020/21 failure to fulfil fixtures</t>
+    <t>Carried over from refusing to play in 2020/21</t>
   </si>
   <si>
     <t>Breach of business plan agreed with the EFL</t>
   </si>
   <si>
     <t>Failure to pay players on time</t>
+  </si>
+  <si>
+    <t>Rule breach (the page gives no detail; implied by the printed points)</t>
   </si>
   <si>
     <t>Breaches of PL profitability and sustainability rules (10 cut to 6 on appeal; then 2 more)</t>
@@ -816,7 +876,7 @@
     <t>Late payment of player wages (suspended deduction activated)</t>
   </si>
   <si>
-    <t>Failure to pay HMRC and players (from memory; not yet verified)</t>
+    <t>Failed to pay debt to HMRC</t>
   </si>
   <si>
     <t>Late transfer payments to other clubs</t>
@@ -828,13 +888,10 @@
     <t>12 administration + 6 payment failures (from memory; not yet verified)</t>
   </si>
   <si>
-    <t>verified</t>
+    <t>Wikipedia final table</t>
   </si>
   <si>
-    <t>check</t>
-  </si>
-  <si>
-    <t>high</t>
+    <t>dragonfootball.co.uk; Wikipedia final table</t>
   </si>
 </sst>
 </file>
@@ -17989,13 +18046,13 @@
         <v>57</v>
       </c>
       <c r="L16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N16">
-        <v>1.23913</v>
+        <v>1.217391</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -44846,7 +44903,7 @@
         <v>14</v>
       </c>
       <c r="C183" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="D183">
         <v>46</v>
@@ -44855,31 +44912,31 @@
         <v>16</v>
       </c>
       <c r="F183">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G183">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H183">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I183">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="J183">
-        <v>-17</v>
+        <v>-6</v>
       </c>
       <c r="K183">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L183">
         <v>0</v>
       </c>
       <c r="M183">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N183">
-        <v>1.304348</v>
+        <v>1.282609</v>
       </c>
     </row>
     <row r="184" spans="1:15">
@@ -44890,7 +44947,7 @@
         <v>15</v>
       </c>
       <c r="C184" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D184">
         <v>46</v>
@@ -44905,13 +44962,13 @@
         <v>19</v>
       </c>
       <c r="H184">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="I184">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="J184">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="K184">
         <v>59</v>
@@ -44934,7 +44991,7 @@
         <v>16</v>
       </c>
       <c r="C185" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="D185">
         <v>46</v>
@@ -44943,31 +45000,31 @@
         <v>16</v>
       </c>
       <c r="F185">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G185">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H185">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="I185">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J185">
-        <v>-7</v>
+        <v>-17</v>
       </c>
       <c r="K185">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="L185">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M185">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N185">
-        <v>1.282609</v>
+        <v>1.23913</v>
       </c>
     </row>
     <row r="186" spans="1:15">
@@ -61472,13 +61529,13 @@
         <v>48</v>
       </c>
       <c r="L121">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M121">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="N121">
-        <v>0.826087</v>
+        <v>1.043478</v>
       </c>
       <c r="O121" t="s">
         <v>76</v>
@@ -75693,40 +75750,40 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="D6">
         <v>46</v>
       </c>
       <c r="E6">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G6">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H6">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I6">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="J6">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K6">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N6">
-        <v>1.782609</v>
+        <v>1.76087</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -75737,7 +75794,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>118</v>
+        <v>150</v>
       </c>
       <c r="D7">
         <v>46</v>
@@ -75746,31 +75803,31 @@
         <v>23</v>
       </c>
       <c r="F7">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G7">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H7">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I7">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="J7">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K7">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="N7">
-        <v>1.76087</v>
+        <v>1.717391</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -75781,40 +75838,40 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>150</v>
+        <v>94</v>
       </c>
       <c r="D8">
         <v>46</v>
       </c>
       <c r="E8">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F8">
         <v>10</v>
       </c>
       <c r="G8">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H8">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I8">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="J8">
         <v>21</v>
       </c>
       <c r="K8">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M8">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="N8">
-        <v>1.717391</v>
+        <v>1.673913</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -75896,13 +75953,13 @@
         <v>71</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N10">
-        <v>1.543478</v>
+        <v>1.521739</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -75957,40 +76014,40 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="D12">
         <v>46</v>
       </c>
       <c r="E12">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F12">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G12">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H12">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="I12">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="K12">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
       <c r="M12">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="N12">
-        <v>1.434783</v>
+        <v>1.369565</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -76001,40 +76058,40 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="D13">
         <v>46</v>
       </c>
       <c r="E13">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F13">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G13">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H13">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="I13">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="J13">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="K13">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="L13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M13">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N13">
-        <v>1.369565</v>
+        <v>1.347826</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -77342,25 +77399,25 @@
         <v>18</v>
       </c>
       <c r="C43" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="D43">
         <v>44</v>
       </c>
       <c r="E43">
+        <v>11</v>
+      </c>
+      <c r="F43">
         <v>13</v>
       </c>
-      <c r="F43">
-        <v>7</v>
-      </c>
       <c r="G43">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H43">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I43">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J43">
         <v>-23</v>
@@ -77386,7 +77443,7 @@
         <v>19</v>
       </c>
       <c r="C44" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D44">
         <v>44</v>
@@ -77401,13 +77458,13 @@
         <v>20</v>
       </c>
       <c r="H44">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I44">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="J44">
-        <v>-23</v>
+        <v>-30</v>
       </c>
       <c r="K44">
         <v>46</v>
@@ -77430,40 +77487,40 @@
         <v>20</v>
       </c>
       <c r="C45" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="D45">
         <v>44</v>
       </c>
       <c r="E45">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F45">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="G45">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H45">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="I45">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="J45">
-        <v>-30</v>
+        <v>-23</v>
       </c>
       <c r="K45">
         <v>46</v>
       </c>
       <c r="L45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M45">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N45">
-        <v>1.045455</v>
+        <v>1.022727</v>
       </c>
     </row>
     <row r="46" spans="1:15">
@@ -77595,13 +77652,13 @@
         <v>28</v>
       </c>
       <c r="L48">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M48">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N48">
-        <v>0.636364</v>
+        <v>0.590909</v>
       </c>
       <c r="O48" t="s">
         <v>76</v>
@@ -78105,43 +78162,40 @@
         <v>12</v>
       </c>
       <c r="C60" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="D60">
         <v>46</v>
       </c>
       <c r="E60">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F60">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G60">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H60">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="I60">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="J60">
-        <v>3</v>
+        <v>-2</v>
       </c>
       <c r="K60">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L60">
         <v>0</v>
       </c>
       <c r="M60">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N60">
-        <v>1.347826</v>
-      </c>
-      <c r="O60" t="s">
-        <v>147</v>
+        <v>1.326087</v>
       </c>
     </row>
     <row r="61" spans="1:15">
@@ -78152,40 +78206,43 @@
         <v>13</v>
       </c>
       <c r="C61" t="s">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="D61">
         <v>46</v>
       </c>
       <c r="E61">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F61">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G61">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H61">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="I61">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="J61">
-        <v>-2</v>
+        <v>3</v>
       </c>
       <c r="K61">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L61">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M61">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="N61">
-        <v>1.326087</v>
+        <v>1.23913</v>
+      </c>
+      <c r="O61" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="62" spans="1:15">
@@ -78196,40 +78253,40 @@
         <v>14</v>
       </c>
       <c r="C62" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="D62">
         <v>46</v>
       </c>
       <c r="E62">
+        <v>14</v>
+      </c>
+      <c r="F62">
         <v>15</v>
       </c>
-      <c r="F62">
-        <v>13</v>
-      </c>
       <c r="G62">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H62">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I62">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="J62">
-        <v>-11</v>
+        <v>-3</v>
       </c>
       <c r="K62">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L62">
         <v>0</v>
       </c>
       <c r="M62">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N62">
-        <v>1.26087</v>
+        <v>1.23913</v>
       </c>
     </row>
     <row r="63" spans="1:15">
@@ -78240,40 +78297,40 @@
         <v>15</v>
       </c>
       <c r="C63" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="D63">
         <v>46</v>
       </c>
       <c r="E63">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F63">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G63">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H63">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I63">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="J63">
-        <v>-3</v>
+        <v>-11</v>
       </c>
       <c r="K63">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L63">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M63">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N63">
-        <v>1.23913</v>
+        <v>1.217391</v>
       </c>
     </row>
     <row r="64" spans="1:15">
@@ -78669,13 +78726,13 @@
         <v>33</v>
       </c>
       <c r="L72">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M72">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="N72">
-        <v>0.717391</v>
+        <v>0.608696</v>
       </c>
       <c r="O72" t="s">
         <v>76</v>
@@ -79669,40 +79726,40 @@
         <v>23</v>
       </c>
       <c r="C95" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="D95">
         <v>46</v>
       </c>
       <c r="E95">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F95">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G95">
         <v>29</v>
       </c>
       <c r="H95">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I95">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="J95">
-        <v>-60</v>
+        <v>-46</v>
       </c>
       <c r="K95">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="L95">
         <v>0</v>
       </c>
       <c r="M95">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="N95">
-        <v>0.717391</v>
+        <v>0.673913</v>
       </c>
       <c r="O95" t="s">
         <v>76</v>
@@ -79716,40 +79773,40 @@
         <v>24</v>
       </c>
       <c r="C96" t="s">
-        <v>165</v>
+        <v>151</v>
       </c>
       <c r="D96">
         <v>46</v>
       </c>
       <c r="E96">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F96">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G96">
         <v>29</v>
       </c>
       <c r="H96">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="I96">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="J96">
-        <v>-46</v>
+        <v>-60</v>
       </c>
       <c r="K96">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L96">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M96">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N96">
-        <v>0.673913</v>
+        <v>0.652174</v>
       </c>
       <c r="O96" t="s">
         <v>76</v>
@@ -81195,40 +81252,40 @@
         <v>9</v>
       </c>
       <c r="C129" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="D129">
         <v>46</v>
       </c>
       <c r="E129">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F129">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G129">
         <v>18</v>
       </c>
       <c r="H129">
+        <v>66</v>
+      </c>
+      <c r="I129">
         <v>69</v>
       </c>
-      <c r="I129">
-        <v>74</v>
-      </c>
       <c r="J129">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="K129">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L129">
         <v>0</v>
       </c>
       <c r="M129">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="N129">
-        <v>1.521739</v>
+        <v>1.478261</v>
       </c>
     </row>
     <row r="130" spans="1:15">
@@ -81239,40 +81296,40 @@
         <v>10</v>
       </c>
       <c r="C130" t="s">
-        <v>158</v>
+        <v>131</v>
       </c>
       <c r="D130">
         <v>46</v>
       </c>
       <c r="E130">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F130">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G130">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H130">
+        <v>80</v>
+      </c>
+      <c r="I130">
         <v>66</v>
       </c>
-      <c r="I130">
-        <v>69</v>
-      </c>
       <c r="J130">
-        <v>-3</v>
+        <v>14</v>
       </c>
       <c r="K130">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L130">
         <v>0</v>
       </c>
       <c r="M130">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N130">
-        <v>1.478261</v>
+        <v>1.456522</v>
       </c>
     </row>
     <row r="131" spans="1:15">
@@ -81283,34 +81340,34 @@
         <v>11</v>
       </c>
       <c r="C131" t="s">
-        <v>131</v>
+        <v>168</v>
       </c>
       <c r="D131">
         <v>46</v>
       </c>
       <c r="E131">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F131">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G131">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H131">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="I131">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="J131">
-        <v>14</v>
+        <v>-5</v>
       </c>
       <c r="K131">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L131">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M131">
         <v>67</v>
@@ -82126,13 +82183,13 @@
         <v>82</v>
       </c>
       <c r="L149">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M149">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="N149">
-        <v>1.782609</v>
+        <v>1.717391</v>
       </c>
     </row>
     <row r="150" spans="1:15">
@@ -82850,28 +82907,28 @@
         <v>22</v>
       </c>
       <c r="C166" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D166">
         <v>46</v>
       </c>
       <c r="E166">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F166">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G166">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H166">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="I166">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="J166">
-        <v>-26</v>
+        <v>-30</v>
       </c>
       <c r="K166">
         <v>39</v>
@@ -82897,40 +82954,40 @@
         <v>23</v>
       </c>
       <c r="C167" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D167">
         <v>46</v>
       </c>
       <c r="E167">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F167">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G167">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="H167">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="I167">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="J167">
-        <v>-30</v>
+        <v>-26</v>
       </c>
       <c r="K167">
         <v>39</v>
       </c>
       <c r="L167">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M167">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="N167">
-        <v>0.847826</v>
+        <v>0.782609</v>
       </c>
       <c r="O167" t="s">
         <v>76</v>
@@ -82971,13 +83028,13 @@
         <v>39</v>
       </c>
       <c r="L168">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M168">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="N168">
-        <v>0.847826</v>
+        <v>0.782609</v>
       </c>
       <c r="O168" t="s">
         <v>76</v>
@@ -86571,43 +86628,40 @@
         <v>9</v>
       </c>
       <c r="C249" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="D249">
         <v>46</v>
       </c>
       <c r="E249">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F249">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G249">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H249">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I249">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="J249">
-        <v>4</v>
+        <v>-5</v>
       </c>
       <c r="K249">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L249">
         <v>0</v>
       </c>
       <c r="M249">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="N249">
-        <v>1.434783</v>
-      </c>
-      <c r="O249" t="s">
-        <v>194</v>
+        <v>1.413043</v>
       </c>
     </row>
     <row r="250" spans="1:15">
@@ -86618,7 +86672,7 @@
         <v>10</v>
       </c>
       <c r="C250" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D250">
         <v>46</v>
@@ -86627,31 +86681,31 @@
         <v>17</v>
       </c>
       <c r="F250">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G250">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H250">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I250">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="J250">
-        <v>-5</v>
+        <v>1</v>
       </c>
       <c r="K250">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L250">
         <v>0</v>
       </c>
       <c r="M250">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N250">
-        <v>1.413043</v>
+        <v>1.391304</v>
       </c>
     </row>
     <row r="251" spans="1:15">
@@ -86662,40 +86716,40 @@
         <v>11</v>
       </c>
       <c r="C251" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D251">
         <v>46</v>
       </c>
       <c r="E251">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F251">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G251">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H251">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="I251">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="J251">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="K251">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="L251">
         <v>0</v>
       </c>
       <c r="M251">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N251">
-        <v>1.391304</v>
+        <v>1.304348</v>
       </c>
     </row>
     <row r="252" spans="1:15">
@@ -86706,7 +86760,7 @@
         <v>12</v>
       </c>
       <c r="C252" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="D252">
         <v>46</v>
@@ -86721,13 +86775,13 @@
         <v>18</v>
       </c>
       <c r="H252">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="I252">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="J252">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="K252">
         <v>60</v>
@@ -86750,7 +86804,7 @@
         <v>13</v>
       </c>
       <c r="C253" t="s">
-        <v>135</v>
+        <v>177</v>
       </c>
       <c r="D253">
         <v>46</v>
@@ -86765,13 +86819,13 @@
         <v>18</v>
       </c>
       <c r="H253">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="I253">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="J253">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="K253">
         <v>60</v>
@@ -86794,40 +86848,40 @@
         <v>14</v>
       </c>
       <c r="C254" t="s">
-        <v>177</v>
+        <v>120</v>
       </c>
       <c r="D254">
         <v>46</v>
       </c>
       <c r="E254">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F254">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G254">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H254">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I254">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="J254">
-        <v>-6</v>
+        <v>2</v>
       </c>
       <c r="K254">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L254">
         <v>0</v>
       </c>
       <c r="M254">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N254">
-        <v>1.304348</v>
+        <v>1.282609</v>
       </c>
     </row>
     <row r="255" spans="1:15">
@@ -86838,28 +86892,28 @@
         <v>15</v>
       </c>
       <c r="C255" t="s">
-        <v>120</v>
+        <v>173</v>
       </c>
       <c r="D255">
         <v>46</v>
       </c>
       <c r="E255">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F255">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G255">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H255">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="I255">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="J255">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K255">
         <v>59</v>
@@ -86882,28 +86936,28 @@
         <v>16</v>
       </c>
       <c r="C256" t="s">
-        <v>173</v>
+        <v>107</v>
       </c>
       <c r="D256">
         <v>46</v>
       </c>
       <c r="E256">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F256">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G256">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H256">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="I256">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="J256">
-        <v>1</v>
+        <v>-6</v>
       </c>
       <c r="K256">
         <v>59</v>
@@ -86926,40 +86980,43 @@
         <v>17</v>
       </c>
       <c r="C257" t="s">
-        <v>107</v>
+        <v>164</v>
       </c>
       <c r="D257">
         <v>46</v>
       </c>
       <c r="E257">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F257">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G257">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H257">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="I257">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="J257">
-        <v>-6</v>
+        <v>4</v>
       </c>
       <c r="K257">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="L257">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="M257">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N257">
-        <v>1.282609</v>
+        <v>1.23913</v>
+      </c>
+      <c r="O257" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="258" spans="1:15">
@@ -87149,40 +87206,40 @@
         <v>22</v>
       </c>
       <c r="C262" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="D262">
         <v>46</v>
       </c>
       <c r="E262">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F262">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G262">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H262">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="I262">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="J262">
-        <v>-30</v>
+        <v>-22</v>
       </c>
       <c r="K262">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L262">
         <v>0</v>
       </c>
       <c r="M262">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N262">
-        <v>0.891304</v>
+        <v>0.869565</v>
       </c>
       <c r="O262" t="s">
         <v>76</v>
@@ -87196,40 +87253,40 @@
         <v>23</v>
       </c>
       <c r="C263" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="D263">
         <v>46</v>
       </c>
       <c r="E263">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F263">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G263">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="H263">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="I263">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="J263">
-        <v>-22</v>
+        <v>-30</v>
       </c>
       <c r="K263">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L263">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M263">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="N263">
-        <v>0.869565</v>
+        <v>0.826087</v>
       </c>
       <c r="O263" t="s">
         <v>76</v>
@@ -90899,28 +90956,28 @@
         <v>13</v>
       </c>
       <c r="C346" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="D346">
         <v>46</v>
       </c>
       <c r="E346">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F346">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G346">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H346">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="I346">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="J346">
-        <v>5</v>
+        <v>-15</v>
       </c>
       <c r="K346">
         <v>60</v>
@@ -90943,40 +91000,40 @@
         <v>14</v>
       </c>
       <c r="C347" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
       <c r="D347">
         <v>46</v>
       </c>
       <c r="E347">
+        <v>15</v>
+      </c>
+      <c r="F347">
+        <v>15</v>
+      </c>
+      <c r="G347">
         <v>16</v>
       </c>
-      <c r="F347">
-        <v>12</v>
-      </c>
-      <c r="G347">
-        <v>18</v>
-      </c>
       <c r="H347">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="I347">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="J347">
-        <v>-15</v>
+        <v>5</v>
       </c>
       <c r="K347">
         <v>60</v>
       </c>
       <c r="L347">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M347">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N347">
-        <v>1.304348</v>
+        <v>1.282609</v>
       </c>
     </row>
     <row r="348" spans="1:14">
@@ -94660,7 +94717,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -94691,7 +94748,7 @@
         <v>2008</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
         <v>202</v>
@@ -94700,13 +94757,13 @@
         <v>11</v>
       </c>
       <c r="E2">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="G2" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -94714,7 +94771,7 @@
         <v>2008</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s">
         <v>203</v>
@@ -94723,13 +94780,13 @@
         <v>11</v>
       </c>
       <c r="E3">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="G3" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -94746,13 +94803,13 @@
         <v>11</v>
       </c>
       <c r="E4">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="G4" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -94769,13 +94826,13 @@
         <v>11</v>
       </c>
       <c r="E5">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="G5" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -94792,21 +94849,21 @@
         <v>11</v>
       </c>
       <c r="E6">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="G6" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7" t="s">
         <v>207</v>
@@ -94815,21 +94872,21 @@
         <v>11</v>
       </c>
       <c r="E7">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="G7" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
         <v>208</v>
@@ -94838,21 +94895,21 @@
         <v>11</v>
       </c>
       <c r="E8">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>238</v>
+        <v>255</v>
       </c>
       <c r="G8" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C9" t="s">
         <v>209</v>
@@ -94861,21 +94918,21 @@
         <v>11</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="G9" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C10" t="s">
         <v>210</v>
@@ -94884,13 +94941,13 @@
         <v>11</v>
       </c>
       <c r="E10">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="G10" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -94898,7 +94955,7 @@
         <v>2009</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C11" t="s">
         <v>211</v>
@@ -94907,13 +94964,13 @@
         <v>11</v>
       </c>
       <c r="E11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F11" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="G11" t="s">
-        <v>270</v>
+        <v>290</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -94921,76 +94978,79 @@
         <v>2009</v>
       </c>
       <c r="B12">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="D12" t="s">
-        <v>237</v>
+        <v>11</v>
+      </c>
+      <c r="E12">
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="G12" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="B13">
         <v>3</v>
       </c>
       <c r="C13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
       </c>
       <c r="E13">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F13" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="G13" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="B14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
       </c>
       <c r="E14">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>241</v>
+        <v>258</v>
       </c>
       <c r="G14" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="B15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -94999,44 +95059,44 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>241</v>
+        <v>259</v>
       </c>
       <c r="G15" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="B16">
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F16" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="G16" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17">
-        <v>2011</v>
+        <v>2009</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -95045,44 +95105,41 @@
         <v>10</v>
       </c>
       <c r="F17" t="s">
-        <v>238</v>
+        <v>261</v>
       </c>
       <c r="G17" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18">
-        <v>2011</v>
+        <v>2009</v>
       </c>
       <c r="B18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C18" t="s">
         <v>217</v>
       </c>
       <c r="D18" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18">
-        <v>10</v>
+        <v>250</v>
       </c>
       <c r="F18" t="s">
-        <v>238</v>
+        <v>262</v>
       </c>
       <c r="G18" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="B19">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -95091,291 +95148,294 @@
         <v>10</v>
       </c>
       <c r="F19" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="G19" t="s">
-        <v>270</v>
+        <v>290</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F20" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="G20" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="B21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
       </c>
       <c r="E21">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="G21" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="B22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="E22">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F22" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="G22" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23">
-        <v>2013</v>
+        <v>2010</v>
       </c>
       <c r="B23">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F23" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G23" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24">
-        <v>2013</v>
+        <v>2010</v>
       </c>
       <c r="B24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F24" t="s">
-        <v>241</v>
+        <v>263</v>
       </c>
       <c r="G24" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25">
-        <v>2013</v>
+        <v>2010</v>
       </c>
       <c r="B25">
         <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="D25" t="s">
         <v>11</v>
       </c>
       <c r="E25">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F25" t="s">
-        <v>249</v>
+        <v>264</v>
       </c>
       <c r="G25" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26">
-        <v>2014</v>
+        <v>2011</v>
       </c>
       <c r="B26">
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="G26" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27">
-        <v>2018</v>
+        <v>2011</v>
       </c>
       <c r="B27">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F27" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G27" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28">
-        <v>2019</v>
+        <v>2011</v>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C28" t="s">
-        <v>222</v>
+        <v>205</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="G28" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29">
-        <v>2019</v>
+        <v>2011</v>
       </c>
       <c r="B29">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F29" t="s">
-        <v>238</v>
+        <v>265</v>
       </c>
       <c r="G29" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="B30">
         <v>3</v>
       </c>
       <c r="C30" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D30" t="s">
-        <v>147</v>
+        <v>11</v>
+      </c>
+      <c r="E30">
+        <v>10</v>
       </c>
       <c r="F30" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G30" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="B31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C31" t="s">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F31" t="s">
         <v>252</v>
       </c>
       <c r="G31" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32">
-        <v>2020</v>
+        <v>2013</v>
       </c>
       <c r="B32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C32" t="s">
         <v>226</v>
@@ -95384,41 +95444,44 @@
         <v>11</v>
       </c>
       <c r="E32">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F32" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="G32" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33">
-        <v>2020</v>
+        <v>2013</v>
       </c>
       <c r="B33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C33" t="s">
         <v>227</v>
       </c>
       <c r="D33" t="s">
-        <v>237</v>
+        <v>11</v>
+      </c>
+      <c r="E33">
+        <v>3</v>
       </c>
       <c r="F33" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="G33" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34">
-        <v>2021</v>
+        <v>2013</v>
       </c>
       <c r="B34">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C34" t="s">
         <v>228</v>
@@ -95427,21 +95490,21 @@
         <v>11</v>
       </c>
       <c r="E34">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F34" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="G34" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35">
-        <v>2021</v>
+        <v>2013</v>
       </c>
       <c r="B35">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
         <v>229</v>
@@ -95450,70 +95513,70 @@
         <v>11</v>
       </c>
       <c r="E35">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F35" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="G35" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36">
-        <v>2021</v>
+        <v>2014</v>
       </c>
       <c r="B36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>227</v>
+        <v>207</v>
       </c>
       <c r="D36" t="s">
         <v>11</v>
       </c>
       <c r="E36">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F36" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="G36" t="s">
-        <v>270</v>
+        <v>290</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37">
-        <v>2022</v>
+        <v>2014</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C37" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F37" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="G37" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="38" spans="1:7">
       <c r="A38">
-        <v>2022</v>
+        <v>2014</v>
       </c>
       <c r="B38">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C38" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
@@ -95522,240 +95585,625 @@
         <v>3</v>
       </c>
       <c r="F38" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="G38" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39">
-        <v>2023</v>
+        <v>2014</v>
       </c>
       <c r="B39">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C39" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F39" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="G39" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40">
-        <v>2023</v>
+        <v>2015</v>
       </c>
       <c r="B40">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C40" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="G40" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="B41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C41" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="E41">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F41" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="G41" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="42" spans="1:7">
       <c r="A42">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="B42">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C42" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F42" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="G42" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="43" spans="1:7">
       <c r="A43">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="B43">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C43" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F43" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="G43" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44">
-        <v>2023</v>
+        <v>2019</v>
       </c>
       <c r="B44">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C44" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
       </c>
       <c r="E44">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F44" t="s">
-        <v>265</v>
+        <v>252</v>
       </c>
       <c r="G44" t="s">
-        <v>270</v>
+        <v>290</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="B45">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C45" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F45" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="G45" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="B46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C46" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D46" t="s">
-        <v>11</v>
-      </c>
-      <c r="E46">
-        <v>6</v>
+        <v>147</v>
       </c>
       <c r="F46" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="G46" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="B47">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C47" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="D47" t="s">
         <v>11</v>
       </c>
       <c r="E47">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F47" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="G47" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="B48">
         <v>2</v>
       </c>
       <c r="C48" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D48" t="s">
         <v>11</v>
       </c>
       <c r="E48">
+        <v>6</v>
+      </c>
+      <c r="F48" t="s">
+        <v>272</v>
+      </c>
+      <c r="G48" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49">
+        <v>2020</v>
+      </c>
+      <c r="B49">
+        <v>5</v>
+      </c>
+      <c r="C49" t="s">
+        <v>240</v>
+      </c>
+      <c r="D49" t="s">
+        <v>250</v>
+      </c>
+      <c r="F49" t="s">
+        <v>273</v>
+      </c>
+      <c r="G49" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50">
+        <v>2021</v>
+      </c>
+      <c r="B50">
         <v>2</v>
       </c>
-      <c r="F48" t="s">
-        <v>256</v>
-      </c>
-      <c r="G48" t="s">
-        <v>269</v>
+      <c r="C50" t="s">
+        <v>241</v>
+      </c>
+      <c r="D50" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50">
+        <v>21</v>
+      </c>
+      <c r="F50" t="s">
+        <v>274</v>
+      </c>
+      <c r="G50" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51">
+        <v>2021</v>
+      </c>
+      <c r="B51">
+        <v>2</v>
+      </c>
+      <c r="C51" t="s">
+        <v>242</v>
+      </c>
+      <c r="D51" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51">
+        <v>6</v>
+      </c>
+      <c r="F51" t="s">
+        <v>275</v>
+      </c>
+      <c r="G51" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52">
+        <v>2021</v>
+      </c>
+      <c r="B52">
+        <v>5</v>
+      </c>
+      <c r="C52" t="s">
+        <v>240</v>
+      </c>
+      <c r="D52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52">
+        <v>12</v>
+      </c>
+      <c r="F52" t="s">
+        <v>276</v>
+      </c>
+      <c r="G52" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53">
+        <v>2022</v>
+      </c>
+      <c r="B53">
+        <v>2</v>
+      </c>
+      <c r="C53" t="s">
+        <v>242</v>
+      </c>
+      <c r="D53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53">
+        <v>6</v>
+      </c>
+      <c r="F53" t="s">
+        <v>277</v>
+      </c>
+      <c r="G53" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54">
+        <v>2022</v>
+      </c>
+      <c r="B54">
+        <v>2</v>
+      </c>
+      <c r="C54" t="s">
+        <v>236</v>
+      </c>
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54">
+        <v>3</v>
+      </c>
+      <c r="F54" t="s">
+        <v>278</v>
+      </c>
+      <c r="G54" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55">
+        <v>2022</v>
+      </c>
+      <c r="B55">
+        <v>5</v>
+      </c>
+      <c r="C55" t="s">
+        <v>214</v>
+      </c>
+      <c r="D55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55" t="s">
+        <v>279</v>
+      </c>
+      <c r="G55" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56">
+        <v>2023</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>243</v>
+      </c>
+      <c r="D56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56">
+        <v>8</v>
+      </c>
+      <c r="F56" t="s">
+        <v>280</v>
+      </c>
+      <c r="G56" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57">
+        <v>2023</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>244</v>
+      </c>
+      <c r="D57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57">
+        <v>4</v>
+      </c>
+      <c r="F57" t="s">
+        <v>281</v>
+      </c>
+      <c r="G57" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58">
+        <v>2023</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>242</v>
+      </c>
+      <c r="D58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58">
+        <v>6</v>
+      </c>
+      <c r="F58" t="s">
+        <v>282</v>
+      </c>
+      <c r="G58" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="A59">
+        <v>2023</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>236</v>
+      </c>
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>283</v>
+      </c>
+      <c r="G59" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="A60">
+        <v>2023</v>
+      </c>
+      <c r="B60">
+        <v>4</v>
+      </c>
+      <c r="C60" t="s">
+        <v>245</v>
+      </c>
+      <c r="D60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60">
+        <v>3</v>
+      </c>
+      <c r="F60" t="s">
+        <v>284</v>
+      </c>
+      <c r="G60" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
+      <c r="A61">
+        <v>2023</v>
+      </c>
+      <c r="B61">
+        <v>5</v>
+      </c>
+      <c r="C61" t="s">
+        <v>246</v>
+      </c>
+      <c r="D61" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61">
+        <v>10</v>
+      </c>
+      <c r="F61" t="s">
+        <v>285</v>
+      </c>
+      <c r="G61" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
+      <c r="A62">
+        <v>2024</v>
+      </c>
+      <c r="B62">
+        <v>2</v>
+      </c>
+      <c r="C62" t="s">
+        <v>247</v>
+      </c>
+      <c r="D62" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62">
+        <v>2</v>
+      </c>
+      <c r="F62" t="s">
+        <v>286</v>
+      </c>
+      <c r="G62" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
+      <c r="A63">
+        <v>2025</v>
+      </c>
+      <c r="B63">
+        <v>2</v>
+      </c>
+      <c r="C63" t="s">
+        <v>248</v>
+      </c>
+      <c r="D63" t="s">
+        <v>11</v>
+      </c>
+      <c r="E63">
+        <v>6</v>
+      </c>
+      <c r="F63" t="s">
+        <v>287</v>
+      </c>
+      <c r="G63" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
+      <c r="A64">
+        <v>2025</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>239</v>
+      </c>
+      <c r="D64" t="s">
+        <v>11</v>
+      </c>
+      <c r="E64">
+        <v>18</v>
+      </c>
+      <c r="F64" t="s">
+        <v>288</v>
+      </c>
+      <c r="G64" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7">
+      <c r="A65">
+        <v>2025</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>249</v>
+      </c>
+      <c r="D65" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65">
+        <v>2</v>
+      </c>
+      <c r="F65" t="s">
+        <v>275</v>
+      </c>
+      <c r="G65" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use football-data as the source of every result
football-data's score now always wins instead of a majority vote, and the
GitHub copy of football-data fills 2013/14 Premier League. engsoccerdata and
openfootball only check it. One result changes: Portsmouth 2-1 Shrewsbury
(2012/13), which moves no points or positions.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S5Qc48tZkYoqs3XftGiQZ8
</commit_message>
<xml_diff>
--- a/data/processed/real_tables.xlsx
+++ b/data/processed/real_tables.xlsx
@@ -41778,10 +41778,10 @@
         <v>54</v>
       </c>
       <c r="I113">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J113">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="K113">
         <v>55</v>
@@ -42136,13 +42136,13 @@
         <v>24</v>
       </c>
       <c r="H121">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I121">
         <v>69</v>
       </c>
       <c r="J121">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="K121">
         <v>42</v>

</xml_diff>